<commit_message>
Add actual M16 signatures per company to unit breakdown sheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HWaTxciq62ssoxtUxBkqgK
</commit_message>
<xml_diff>
--- a/count_report_2026-07-05.xlsx
+++ b/count_report_2026-07-05.xlsx
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +187,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1948,7 +1954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2769,11 +2775,81 @@
         <v>1</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>M16 (חתום בפועל)</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="15" t="n">
+        <v>33</v>
+      </c>
+      <c r="K21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>סה"כ 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>* M16 אינו מוקצה לפלוגות (מנוהל ברמת הגדוד) – השורה מציגה חתימות בפועל לפי דוח החתימות האישי; עוד 132 במלאי הגדודי.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A22:N22"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="A3:A4"/>
@@ -2787,6 +2863,8 @@
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0.75</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N5:N22">
     <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="2">
       <formula>0.9</formula>
     </cfRule>
@@ -2828,32 +2906,32 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>שם פריט</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>פלוגה א</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
+      <c r="D3" s="26" t="inlineStr">
         <is>
           <t>פלוגה ב</t>
         </is>
       </c>
-      <c r="F3" s="24" t="inlineStr">
+      <c r="F3" s="26" t="inlineStr">
         <is>
           <t>פלוגה ג</t>
         </is>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="26" t="inlineStr">
         <is>
           <t>מסייעת</t>
         </is>
       </c>
-      <c r="J3" s="24" t="inlineStr">
+      <c r="J3" s="26" t="inlineStr">
         <is>
           <t>פלס"ם</t>
         </is>

</xml_diff>